<commit_message>
Pflege & Hosting mit 12 Monaten Laufzeit (verlängert sich jährlich) statt monatlich kündbar – Website, FAQ, Preise, Businessplan, Finanzmodell
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LjBk9rJLZKY7FRamo8XJBR
</commit_message>
<xml_diff>
--- a/finanzen/Finanzmodell.xlsx
+++ b/finanzen/Finanzmodell.xlsx
@@ -217,13 +217,13 @@
     <t xml:space="preserve">Pflege &amp; Hosting Start</t>
   </si>
   <si>
-    <t xml:space="preserve">monatlich kündbar</t>
+    <t xml:space="preserve">12 Monate Laufzeit</t>
   </si>
   <si>
     <t xml:space="preserve">Pflege &amp; Hosting Wachstum</t>
   </si>
   <si>
-    <t xml:space="preserve">inkl. 1 h Änderungen</t>
+    <t xml:space="preserve">12 Monate Laufzeit, inkl. 1 h Änderungen</t>
   </si>
   <si>
     <t xml:space="preserve">SEO Lokal</t>
@@ -1670,11 +1670,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="31234482"/>
-        <c:axId val="88360962"/>
+        <c:axId val="47329462"/>
+        <c:axId val="18145642"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="31234482"/>
+        <c:axId val="47329462"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1740,7 +1740,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88360962"/>
+        <c:crossAx val="18145642"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1748,7 +1748,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="88360962"/>
+        <c:axId val="18145642"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1824,7 +1824,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31234482"/>
+        <c:crossAx val="47329462"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Preise: Website Start 1.790, Wachstum 3.490, Wachstumsprogramm 1.390/Monat; Recruiting-Werbebudget klar als zusätzlich ausgewiesen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Mzrs4dTG7G67Xhav2xc6z
</commit_message>
<xml_diff>
--- a/finanzen/Finanzmodell.xlsx
+++ b/finanzen/Finanzmodell.xlsx
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="B14" s="10">
-        <f>"Jun 27"</f>
+        <f>"Mai 27"</f>
         <v/>
       </c>
       <c r="C14" s="2" t="n"/>
@@ -2031,62 +2031,62 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
+          <t>Mai 27</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
           <t>Jun 27</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Jul 27</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Aug 27</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Sep 27</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Okt 27</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Nov 27</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Dez 27</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Jan 28</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Feb 28</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Mär 28</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>Apr 28</t>
-        </is>
-      </c>
-      <c r="P4" s="4" t="inlineStr">
-        <is>
-          <t>Mai 28</t>
         </is>
       </c>
       <c r="Q4" s="4" t="inlineStr">
@@ -2102,7 +2102,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>2600</v>
+        <v>3050</v>
       </c>
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="5" t="inlineStr">
@@ -2403,7 +2403,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>1190</v>
+        <v>1390</v>
       </c>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="7" t="inlineStr">
@@ -4630,7 +4630,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>1490</v>
+        <v>1790</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>0</v>
@@ -4666,7 +4666,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>2990</v>
+        <v>3490</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>0</v>
@@ -4921,7 +4921,7 @@
         <v>1490</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>1190</v>
+        <v>1390</v>
       </c>
       <c r="D14" s="13" t="n">
         <v>28</v>
@@ -5040,7 +5040,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>2200</v>
+        <v>2600</v>
       </c>
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="n"/>
@@ -5064,7 +5064,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>1190</v>
+        <v>1390</v>
       </c>
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n"/>

</xml_diff>

<commit_message>
Recruiting Basis (990 € + 490 €/Monat, 1 Stelle, ohne Garantie) neben Recruiting Komplett; Steuerzentrale: aktuelle Preise
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Mzrs4dTG7G67Xhav2xc6z
</commit_message>
<xml_diff>
--- a/finanzen/Finanzmodell.xlsx
+++ b/finanzen/Finanzmodell.xlsx
@@ -4504,7 +4504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4878,20 +4878,20 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Recruiting-Paket</t>
+          <t>Recruiting Basis</t>
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>1490</v>
+        <v>990</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>790</v>
+        <v>490</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F13" s="14">
         <f>B13+12*C13</f>
@@ -4907,27 +4907,27 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>zzgl. Werbebudget, 3 Monate Mindestlaufzeit</t>
+          <t>1 Stelle, zzgl. Werbebudget, 3 Monate Mindestlaufzeit</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Wachstumsprogramm</t>
+          <t>Recruiting Komplett</t>
         </is>
       </c>
       <c r="B14" s="12" t="n">
         <v>1490</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>1390</v>
+        <v>790</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="E14" s="13" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F14" s="14">
         <f>B14+12*C14</f>
@@ -4943,27 +4943,48 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
+          <t>zzgl. Werbebudget, 3 Monate Mindestlaufzeit, mit Garantie</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Wachstumsprogramm</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>1490</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>1390</v>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>28</v>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="F15" s="14">
+        <f>B15+12*C15</f>
+        <v/>
+      </c>
+      <c r="G15" s="15">
+        <f>D15+12*E15+$B$3</f>
+        <v/>
+      </c>
+      <c r="H15" s="16">
+        <f>IF(G15&gt;0,F15/G15,0)</f>
+        <v/>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
           <t>12 Monate, Website + SEO Plus + Ads inklusive</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-    </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Faustregel netto: Vom Gewinn 35–40 % für Einkommensteuer und Sozialversicherung zurücklegen (Steuerberater fragen).</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="n"/>
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="n"/>
@@ -4972,6 +4993,21 @@
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Faustregel netto: Vom Gewinn 35–40 % für Einkommensteuer und Sozialversicherung zurücklegen (Steuerberater fragen).</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Recruiting: Mindestlaufzeit 1 Monat, Bewerbungs-Garantie gestrichen (Website, AGB, Handbuch, Steuerzentrale, Finanzmodell)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Mzrs4dTG7G67Xhav2xc6z
</commit_message>
<xml_diff>
--- a/finanzen/Finanzmodell.xlsx
+++ b/finanzen/Finanzmodell.xlsx
@@ -4907,7 +4907,7 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>1 Stelle, zzgl. Werbebudget, 3 Monate Mindestlaufzeit</t>
+          <t>1 Stelle, zzgl. Werbebudget, 1 Monat Mindestlaufzeit</t>
         </is>
       </c>
     </row>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>zzgl. Werbebudget, 3 Monate Mindestlaufzeit, mit Garantie</t>
+          <t>zzgl. Werbebudget, 1 Monat Mindestlaufzeit</t>
         </is>
       </c>
     </row>

</xml_diff>